<commit_message>
Planner v1.1: track gifts and thank-yous in the guest list
Adds Dar and Poděkováno columns at the end of the guest sheet so
existing formulas are untouched; recalculated with 0 formula errors and
the dashboard totals are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4ZDnfkuU5cm6b5gWA3X3Y
</commit_message>
<xml_diff>
--- a/product/dist/svatebni-planovac-anoberu.xlsx
+++ b/product/dist/svatebni-planovac-anoberu.xlsx
@@ -5931,7 +5931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M254"/>
+  <dimension ref="A1:O254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5947,6 +5947,8 @@
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -6029,6 +6031,16 @@
           <t>Poznámka</t>
         </is>
       </c>
+      <c r="N4" s="22" t="inlineStr">
+        <is>
+          <t>Dar (po svatbě)</t>
+        </is>
+      </c>
+      <c r="O4" s="23" t="inlineStr">
+        <is>
+          <t>Poděkováno</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="24" t="inlineStr">
@@ -6084,6 +6096,8 @@
           <t>příklad – přepište nebo smažte</t>
         </is>
       </c>
+      <c r="N5" s="24" t="n"/>
+      <c r="O5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="24" t="n"/>
@@ -6099,6 +6113,8 @@
       <c r="K6" s="25" t="n"/>
       <c r="L6" s="24" t="n"/>
       <c r="M6" s="24" t="n"/>
+      <c r="N6" s="24" t="n"/>
+      <c r="O6" s="27" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="24" t="n"/>
@@ -6114,6 +6130,8 @@
       <c r="K7" s="25" t="n"/>
       <c r="L7" s="24" t="n"/>
       <c r="M7" s="24" t="n"/>
+      <c r="N7" s="24" t="n"/>
+      <c r="O7" s="27" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="24" t="n"/>
@@ -6129,6 +6147,8 @@
       <c r="K8" s="25" t="n"/>
       <c r="L8" s="24" t="n"/>
       <c r="M8" s="24" t="n"/>
+      <c r="N8" s="24" t="n"/>
+      <c r="O8" s="27" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="24" t="n"/>
@@ -6144,6 +6164,8 @@
       <c r="K9" s="25" t="n"/>
       <c r="L9" s="24" t="n"/>
       <c r="M9" s="24" t="n"/>
+      <c r="N9" s="24" t="n"/>
+      <c r="O9" s="27" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="24" t="n"/>
@@ -6159,6 +6181,8 @@
       <c r="K10" s="25" t="n"/>
       <c r="L10" s="24" t="n"/>
       <c r="M10" s="24" t="n"/>
+      <c r="N10" s="24" t="n"/>
+      <c r="O10" s="27" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="24" t="n"/>
@@ -6174,6 +6198,8 @@
       <c r="K11" s="25" t="n"/>
       <c r="L11" s="24" t="n"/>
       <c r="M11" s="24" t="n"/>
+      <c r="N11" s="24" t="n"/>
+      <c r="O11" s="27" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="24" t="n"/>
@@ -6189,6 +6215,8 @@
       <c r="K12" s="25" t="n"/>
       <c r="L12" s="24" t="n"/>
       <c r="M12" s="24" t="n"/>
+      <c r="N12" s="24" t="n"/>
+      <c r="O12" s="27" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="24" t="n"/>
@@ -6204,6 +6232,8 @@
       <c r="K13" s="25" t="n"/>
       <c r="L13" s="24" t="n"/>
       <c r="M13" s="24" t="n"/>
+      <c r="N13" s="24" t="n"/>
+      <c r="O13" s="27" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="24" t="n"/>
@@ -6219,6 +6249,8 @@
       <c r="K14" s="25" t="n"/>
       <c r="L14" s="24" t="n"/>
       <c r="M14" s="24" t="n"/>
+      <c r="N14" s="24" t="n"/>
+      <c r="O14" s="27" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="24" t="n"/>
@@ -6234,6 +6266,8 @@
       <c r="K15" s="25" t="n"/>
       <c r="L15" s="24" t="n"/>
       <c r="M15" s="24" t="n"/>
+      <c r="N15" s="24" t="n"/>
+      <c r="O15" s="27" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="24" t="n"/>
@@ -6249,6 +6283,8 @@
       <c r="K16" s="25" t="n"/>
       <c r="L16" s="24" t="n"/>
       <c r="M16" s="24" t="n"/>
+      <c r="N16" s="24" t="n"/>
+      <c r="O16" s="27" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="24" t="n"/>
@@ -6264,6 +6300,8 @@
       <c r="K17" s="25" t="n"/>
       <c r="L17" s="24" t="n"/>
       <c r="M17" s="24" t="n"/>
+      <c r="N17" s="24" t="n"/>
+      <c r="O17" s="27" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="24" t="n"/>
@@ -6279,6 +6317,8 @@
       <c r="K18" s="25" t="n"/>
       <c r="L18" s="24" t="n"/>
       <c r="M18" s="24" t="n"/>
+      <c r="N18" s="24" t="n"/>
+      <c r="O18" s="27" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="24" t="n"/>
@@ -6294,6 +6334,8 @@
       <c r="K19" s="25" t="n"/>
       <c r="L19" s="24" t="n"/>
       <c r="M19" s="24" t="n"/>
+      <c r="N19" s="24" t="n"/>
+      <c r="O19" s="27" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="24" t="n"/>
@@ -6309,6 +6351,8 @@
       <c r="K20" s="25" t="n"/>
       <c r="L20" s="24" t="n"/>
       <c r="M20" s="24" t="n"/>
+      <c r="N20" s="24" t="n"/>
+      <c r="O20" s="27" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="24" t="n"/>
@@ -6324,6 +6368,8 @@
       <c r="K21" s="25" t="n"/>
       <c r="L21" s="24" t="n"/>
       <c r="M21" s="24" t="n"/>
+      <c r="N21" s="24" t="n"/>
+      <c r="O21" s="27" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="24" t="n"/>
@@ -6339,6 +6385,8 @@
       <c r="K22" s="25" t="n"/>
       <c r="L22" s="24" t="n"/>
       <c r="M22" s="24" t="n"/>
+      <c r="N22" s="24" t="n"/>
+      <c r="O22" s="27" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="24" t="n"/>
@@ -6354,6 +6402,8 @@
       <c r="K23" s="25" t="n"/>
       <c r="L23" s="24" t="n"/>
       <c r="M23" s="24" t="n"/>
+      <c r="N23" s="24" t="n"/>
+      <c r="O23" s="27" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="24" t="n"/>
@@ -6369,6 +6419,8 @@
       <c r="K24" s="25" t="n"/>
       <c r="L24" s="24" t="n"/>
       <c r="M24" s="24" t="n"/>
+      <c r="N24" s="24" t="n"/>
+      <c r="O24" s="27" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="24" t="n"/>
@@ -6384,6 +6436,8 @@
       <c r="K25" s="25" t="n"/>
       <c r="L25" s="24" t="n"/>
       <c r="M25" s="24" t="n"/>
+      <c r="N25" s="24" t="n"/>
+      <c r="O25" s="27" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="24" t="n"/>
@@ -6399,6 +6453,8 @@
       <c r="K26" s="25" t="n"/>
       <c r="L26" s="24" t="n"/>
       <c r="M26" s="24" t="n"/>
+      <c r="N26" s="24" t="n"/>
+      <c r="O26" s="27" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="24" t="n"/>
@@ -6414,6 +6470,8 @@
       <c r="K27" s="25" t="n"/>
       <c r="L27" s="24" t="n"/>
       <c r="M27" s="24" t="n"/>
+      <c r="N27" s="24" t="n"/>
+      <c r="O27" s="27" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="24" t="n"/>
@@ -6429,6 +6487,8 @@
       <c r="K28" s="25" t="n"/>
       <c r="L28" s="24" t="n"/>
       <c r="M28" s="24" t="n"/>
+      <c r="N28" s="24" t="n"/>
+      <c r="O28" s="27" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="24" t="n"/>
@@ -6444,6 +6504,8 @@
       <c r="K29" s="25" t="n"/>
       <c r="L29" s="24" t="n"/>
       <c r="M29" s="24" t="n"/>
+      <c r="N29" s="24" t="n"/>
+      <c r="O29" s="27" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="24" t="n"/>
@@ -6459,6 +6521,8 @@
       <c r="K30" s="25" t="n"/>
       <c r="L30" s="24" t="n"/>
       <c r="M30" s="24" t="n"/>
+      <c r="N30" s="24" t="n"/>
+      <c r="O30" s="27" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="24" t="n"/>
@@ -6474,6 +6538,8 @@
       <c r="K31" s="25" t="n"/>
       <c r="L31" s="24" t="n"/>
       <c r="M31" s="24" t="n"/>
+      <c r="N31" s="24" t="n"/>
+      <c r="O31" s="27" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="24" t="n"/>
@@ -6489,6 +6555,8 @@
       <c r="K32" s="25" t="n"/>
       <c r="L32" s="24" t="n"/>
       <c r="M32" s="24" t="n"/>
+      <c r="N32" s="24" t="n"/>
+      <c r="O32" s="27" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="24" t="n"/>
@@ -6504,6 +6572,8 @@
       <c r="K33" s="25" t="n"/>
       <c r="L33" s="24" t="n"/>
       <c r="M33" s="24" t="n"/>
+      <c r="N33" s="24" t="n"/>
+      <c r="O33" s="27" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="24" t="n"/>
@@ -6519,6 +6589,8 @@
       <c r="K34" s="25" t="n"/>
       <c r="L34" s="24" t="n"/>
       <c r="M34" s="24" t="n"/>
+      <c r="N34" s="24" t="n"/>
+      <c r="O34" s="27" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="24" t="n"/>
@@ -6534,6 +6606,8 @@
       <c r="K35" s="25" t="n"/>
       <c r="L35" s="24" t="n"/>
       <c r="M35" s="24" t="n"/>
+      <c r="N35" s="24" t="n"/>
+      <c r="O35" s="27" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="24" t="n"/>
@@ -6549,6 +6623,8 @@
       <c r="K36" s="25" t="n"/>
       <c r="L36" s="24" t="n"/>
       <c r="M36" s="24" t="n"/>
+      <c r="N36" s="24" t="n"/>
+      <c r="O36" s="27" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="24" t="n"/>
@@ -6564,6 +6640,8 @@
       <c r="K37" s="25" t="n"/>
       <c r="L37" s="24" t="n"/>
       <c r="M37" s="24" t="n"/>
+      <c r="N37" s="24" t="n"/>
+      <c r="O37" s="27" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="24" t="n"/>
@@ -6579,6 +6657,8 @@
       <c r="K38" s="25" t="n"/>
       <c r="L38" s="24" t="n"/>
       <c r="M38" s="24" t="n"/>
+      <c r="N38" s="24" t="n"/>
+      <c r="O38" s="27" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="24" t="n"/>
@@ -6594,6 +6674,8 @@
       <c r="K39" s="25" t="n"/>
       <c r="L39" s="24" t="n"/>
       <c r="M39" s="24" t="n"/>
+      <c r="N39" s="24" t="n"/>
+      <c r="O39" s="27" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="24" t="n"/>
@@ -6609,6 +6691,8 @@
       <c r="K40" s="25" t="n"/>
       <c r="L40" s="24" t="n"/>
       <c r="M40" s="24" t="n"/>
+      <c r="N40" s="24" t="n"/>
+      <c r="O40" s="27" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="24" t="n"/>
@@ -6624,6 +6708,8 @@
       <c r="K41" s="25" t="n"/>
       <c r="L41" s="24" t="n"/>
       <c r="M41" s="24" t="n"/>
+      <c r="N41" s="24" t="n"/>
+      <c r="O41" s="27" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="24" t="n"/>
@@ -6639,6 +6725,8 @@
       <c r="K42" s="25" t="n"/>
       <c r="L42" s="24" t="n"/>
       <c r="M42" s="24" t="n"/>
+      <c r="N42" s="24" t="n"/>
+      <c r="O42" s="27" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="24" t="n"/>
@@ -6654,6 +6742,8 @@
       <c r="K43" s="25" t="n"/>
       <c r="L43" s="24" t="n"/>
       <c r="M43" s="24" t="n"/>
+      <c r="N43" s="24" t="n"/>
+      <c r="O43" s="27" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="24" t="n"/>
@@ -6669,6 +6759,8 @@
       <c r="K44" s="25" t="n"/>
       <c r="L44" s="24" t="n"/>
       <c r="M44" s="24" t="n"/>
+      <c r="N44" s="24" t="n"/>
+      <c r="O44" s="27" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="24" t="n"/>
@@ -6684,6 +6776,8 @@
       <c r="K45" s="25" t="n"/>
       <c r="L45" s="24" t="n"/>
       <c r="M45" s="24" t="n"/>
+      <c r="N45" s="24" t="n"/>
+      <c r="O45" s="27" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="24" t="n"/>
@@ -6699,6 +6793,8 @@
       <c r="K46" s="25" t="n"/>
       <c r="L46" s="24" t="n"/>
       <c r="M46" s="24" t="n"/>
+      <c r="N46" s="24" t="n"/>
+      <c r="O46" s="27" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="24" t="n"/>
@@ -6714,6 +6810,8 @@
       <c r="K47" s="25" t="n"/>
       <c r="L47" s="24" t="n"/>
       <c r="M47" s="24" t="n"/>
+      <c r="N47" s="24" t="n"/>
+      <c r="O47" s="27" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="24" t="n"/>
@@ -6729,6 +6827,8 @@
       <c r="K48" s="25" t="n"/>
       <c r="L48" s="24" t="n"/>
       <c r="M48" s="24" t="n"/>
+      <c r="N48" s="24" t="n"/>
+      <c r="O48" s="27" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="24" t="n"/>
@@ -6744,6 +6844,8 @@
       <c r="K49" s="25" t="n"/>
       <c r="L49" s="24" t="n"/>
       <c r="M49" s="24" t="n"/>
+      <c r="N49" s="24" t="n"/>
+      <c r="O49" s="27" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="24" t="n"/>
@@ -6759,6 +6861,8 @@
       <c r="K50" s="25" t="n"/>
       <c r="L50" s="24" t="n"/>
       <c r="M50" s="24" t="n"/>
+      <c r="N50" s="24" t="n"/>
+      <c r="O50" s="27" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="24" t="n"/>
@@ -6774,6 +6878,8 @@
       <c r="K51" s="25" t="n"/>
       <c r="L51" s="24" t="n"/>
       <c r="M51" s="24" t="n"/>
+      <c r="N51" s="24" t="n"/>
+      <c r="O51" s="27" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="24" t="n"/>
@@ -6789,6 +6895,8 @@
       <c r="K52" s="25" t="n"/>
       <c r="L52" s="24" t="n"/>
       <c r="M52" s="24" t="n"/>
+      <c r="N52" s="24" t="n"/>
+      <c r="O52" s="27" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="24" t="n"/>
@@ -6804,6 +6912,8 @@
       <c r="K53" s="25" t="n"/>
       <c r="L53" s="24" t="n"/>
       <c r="M53" s="24" t="n"/>
+      <c r="N53" s="24" t="n"/>
+      <c r="O53" s="27" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="24" t="n"/>
@@ -6819,6 +6929,8 @@
       <c r="K54" s="25" t="n"/>
       <c r="L54" s="24" t="n"/>
       <c r="M54" s="24" t="n"/>
+      <c r="N54" s="24" t="n"/>
+      <c r="O54" s="27" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="24" t="n"/>
@@ -6834,6 +6946,8 @@
       <c r="K55" s="25" t="n"/>
       <c r="L55" s="24" t="n"/>
       <c r="M55" s="24" t="n"/>
+      <c r="N55" s="24" t="n"/>
+      <c r="O55" s="27" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="24" t="n"/>
@@ -6849,6 +6963,8 @@
       <c r="K56" s="25" t="n"/>
       <c r="L56" s="24" t="n"/>
       <c r="M56" s="24" t="n"/>
+      <c r="N56" s="24" t="n"/>
+      <c r="O56" s="27" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="24" t="n"/>
@@ -6864,6 +6980,8 @@
       <c r="K57" s="25" t="n"/>
       <c r="L57" s="24" t="n"/>
       <c r="M57" s="24" t="n"/>
+      <c r="N57" s="24" t="n"/>
+      <c r="O57" s="27" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="24" t="n"/>
@@ -6879,6 +6997,8 @@
       <c r="K58" s="25" t="n"/>
       <c r="L58" s="24" t="n"/>
       <c r="M58" s="24" t="n"/>
+      <c r="N58" s="24" t="n"/>
+      <c r="O58" s="27" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="24" t="n"/>
@@ -6894,6 +7014,8 @@
       <c r="K59" s="25" t="n"/>
       <c r="L59" s="24" t="n"/>
       <c r="M59" s="24" t="n"/>
+      <c r="N59" s="24" t="n"/>
+      <c r="O59" s="27" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="24" t="n"/>
@@ -6909,6 +7031,8 @@
       <c r="K60" s="25" t="n"/>
       <c r="L60" s="24" t="n"/>
       <c r="M60" s="24" t="n"/>
+      <c r="N60" s="24" t="n"/>
+      <c r="O60" s="27" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="24" t="n"/>
@@ -6924,6 +7048,8 @@
       <c r="K61" s="25" t="n"/>
       <c r="L61" s="24" t="n"/>
       <c r="M61" s="24" t="n"/>
+      <c r="N61" s="24" t="n"/>
+      <c r="O61" s="27" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="24" t="n"/>
@@ -6939,6 +7065,8 @@
       <c r="K62" s="25" t="n"/>
       <c r="L62" s="24" t="n"/>
       <c r="M62" s="24" t="n"/>
+      <c r="N62" s="24" t="n"/>
+      <c r="O62" s="27" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="24" t="n"/>
@@ -6954,6 +7082,8 @@
       <c r="K63" s="25" t="n"/>
       <c r="L63" s="24" t="n"/>
       <c r="M63" s="24" t="n"/>
+      <c r="N63" s="24" t="n"/>
+      <c r="O63" s="27" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="24" t="n"/>
@@ -6969,6 +7099,8 @@
       <c r="K64" s="25" t="n"/>
       <c r="L64" s="24" t="n"/>
       <c r="M64" s="24" t="n"/>
+      <c r="N64" s="24" t="n"/>
+      <c r="O64" s="27" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="24" t="n"/>
@@ -6984,6 +7116,8 @@
       <c r="K65" s="25" t="n"/>
       <c r="L65" s="24" t="n"/>
       <c r="M65" s="24" t="n"/>
+      <c r="N65" s="24" t="n"/>
+      <c r="O65" s="27" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="24" t="n"/>
@@ -6999,6 +7133,8 @@
       <c r="K66" s="25" t="n"/>
       <c r="L66" s="24" t="n"/>
       <c r="M66" s="24" t="n"/>
+      <c r="N66" s="24" t="n"/>
+      <c r="O66" s="27" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="24" t="n"/>
@@ -7014,6 +7150,8 @@
       <c r="K67" s="25" t="n"/>
       <c r="L67" s="24" t="n"/>
       <c r="M67" s="24" t="n"/>
+      <c r="N67" s="24" t="n"/>
+      <c r="O67" s="27" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="24" t="n"/>
@@ -7029,6 +7167,8 @@
       <c r="K68" s="25" t="n"/>
       <c r="L68" s="24" t="n"/>
       <c r="M68" s="24" t="n"/>
+      <c r="N68" s="24" t="n"/>
+      <c r="O68" s="27" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="24" t="n"/>
@@ -7044,6 +7184,8 @@
       <c r="K69" s="25" t="n"/>
       <c r="L69" s="24" t="n"/>
       <c r="M69" s="24" t="n"/>
+      <c r="N69" s="24" t="n"/>
+      <c r="O69" s="27" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="24" t="n"/>
@@ -7059,6 +7201,8 @@
       <c r="K70" s="25" t="n"/>
       <c r="L70" s="24" t="n"/>
       <c r="M70" s="24" t="n"/>
+      <c r="N70" s="24" t="n"/>
+      <c r="O70" s="27" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="24" t="n"/>
@@ -7074,6 +7218,8 @@
       <c r="K71" s="25" t="n"/>
       <c r="L71" s="24" t="n"/>
       <c r="M71" s="24" t="n"/>
+      <c r="N71" s="24" t="n"/>
+      <c r="O71" s="27" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="24" t="n"/>
@@ -7089,6 +7235,8 @@
       <c r="K72" s="25" t="n"/>
       <c r="L72" s="24" t="n"/>
       <c r="M72" s="24" t="n"/>
+      <c r="N72" s="24" t="n"/>
+      <c r="O72" s="27" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="24" t="n"/>
@@ -7104,6 +7252,8 @@
       <c r="K73" s="25" t="n"/>
       <c r="L73" s="24" t="n"/>
       <c r="M73" s="24" t="n"/>
+      <c r="N73" s="24" t="n"/>
+      <c r="O73" s="27" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="24" t="n"/>
@@ -7119,6 +7269,8 @@
       <c r="K74" s="25" t="n"/>
       <c r="L74" s="24" t="n"/>
       <c r="M74" s="24" t="n"/>
+      <c r="N74" s="24" t="n"/>
+      <c r="O74" s="27" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="24" t="n"/>
@@ -7134,6 +7286,8 @@
       <c r="K75" s="25" t="n"/>
       <c r="L75" s="24" t="n"/>
       <c r="M75" s="24" t="n"/>
+      <c r="N75" s="24" t="n"/>
+      <c r="O75" s="27" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="24" t="n"/>
@@ -7149,6 +7303,8 @@
       <c r="K76" s="25" t="n"/>
       <c r="L76" s="24" t="n"/>
       <c r="M76" s="24" t="n"/>
+      <c r="N76" s="24" t="n"/>
+      <c r="O76" s="27" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="24" t="n"/>
@@ -7164,6 +7320,8 @@
       <c r="K77" s="25" t="n"/>
       <c r="L77" s="24" t="n"/>
       <c r="M77" s="24" t="n"/>
+      <c r="N77" s="24" t="n"/>
+      <c r="O77" s="27" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="24" t="n"/>
@@ -7179,6 +7337,8 @@
       <c r="K78" s="25" t="n"/>
       <c r="L78" s="24" t="n"/>
       <c r="M78" s="24" t="n"/>
+      <c r="N78" s="24" t="n"/>
+      <c r="O78" s="27" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="24" t="n"/>
@@ -7194,6 +7354,8 @@
       <c r="K79" s="25" t="n"/>
       <c r="L79" s="24" t="n"/>
       <c r="M79" s="24" t="n"/>
+      <c r="N79" s="24" t="n"/>
+      <c r="O79" s="27" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="24" t="n"/>
@@ -7209,6 +7371,8 @@
       <c r="K80" s="25" t="n"/>
       <c r="L80" s="24" t="n"/>
       <c r="M80" s="24" t="n"/>
+      <c r="N80" s="24" t="n"/>
+      <c r="O80" s="27" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="24" t="n"/>
@@ -7224,6 +7388,8 @@
       <c r="K81" s="25" t="n"/>
       <c r="L81" s="24" t="n"/>
       <c r="M81" s="24" t="n"/>
+      <c r="N81" s="24" t="n"/>
+      <c r="O81" s="27" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="24" t="n"/>
@@ -7239,6 +7405,8 @@
       <c r="K82" s="25" t="n"/>
       <c r="L82" s="24" t="n"/>
       <c r="M82" s="24" t="n"/>
+      <c r="N82" s="24" t="n"/>
+      <c r="O82" s="27" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="24" t="n"/>
@@ -7254,6 +7422,8 @@
       <c r="K83" s="25" t="n"/>
       <c r="L83" s="24" t="n"/>
       <c r="M83" s="24" t="n"/>
+      <c r="N83" s="24" t="n"/>
+      <c r="O83" s="27" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="24" t="n"/>
@@ -7269,6 +7439,8 @@
       <c r="K84" s="25" t="n"/>
       <c r="L84" s="24" t="n"/>
       <c r="M84" s="24" t="n"/>
+      <c r="N84" s="24" t="n"/>
+      <c r="O84" s="27" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="24" t="n"/>
@@ -7284,6 +7456,8 @@
       <c r="K85" s="25" t="n"/>
       <c r="L85" s="24" t="n"/>
       <c r="M85" s="24" t="n"/>
+      <c r="N85" s="24" t="n"/>
+      <c r="O85" s="27" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="24" t="n"/>
@@ -7299,6 +7473,8 @@
       <c r="K86" s="25" t="n"/>
       <c r="L86" s="24" t="n"/>
       <c r="M86" s="24" t="n"/>
+      <c r="N86" s="24" t="n"/>
+      <c r="O86" s="27" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="24" t="n"/>
@@ -7314,6 +7490,8 @@
       <c r="K87" s="25" t="n"/>
       <c r="L87" s="24" t="n"/>
       <c r="M87" s="24" t="n"/>
+      <c r="N87" s="24" t="n"/>
+      <c r="O87" s="27" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="24" t="n"/>
@@ -7329,6 +7507,8 @@
       <c r="K88" s="25" t="n"/>
       <c r="L88" s="24" t="n"/>
       <c r="M88" s="24" t="n"/>
+      <c r="N88" s="24" t="n"/>
+      <c r="O88" s="27" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="24" t="n"/>
@@ -7344,6 +7524,8 @@
       <c r="K89" s="25" t="n"/>
       <c r="L89" s="24" t="n"/>
       <c r="M89" s="24" t="n"/>
+      <c r="N89" s="24" t="n"/>
+      <c r="O89" s="27" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="24" t="n"/>
@@ -7359,6 +7541,8 @@
       <c r="K90" s="25" t="n"/>
       <c r="L90" s="24" t="n"/>
       <c r="M90" s="24" t="n"/>
+      <c r="N90" s="24" t="n"/>
+      <c r="O90" s="27" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="24" t="n"/>
@@ -7374,6 +7558,8 @@
       <c r="K91" s="25" t="n"/>
       <c r="L91" s="24" t="n"/>
       <c r="M91" s="24" t="n"/>
+      <c r="N91" s="24" t="n"/>
+      <c r="O91" s="27" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="24" t="n"/>
@@ -7389,6 +7575,8 @@
       <c r="K92" s="25" t="n"/>
       <c r="L92" s="24" t="n"/>
       <c r="M92" s="24" t="n"/>
+      <c r="N92" s="24" t="n"/>
+      <c r="O92" s="27" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="24" t="n"/>
@@ -7404,6 +7592,8 @@
       <c r="K93" s="25" t="n"/>
       <c r="L93" s="24" t="n"/>
       <c r="M93" s="24" t="n"/>
+      <c r="N93" s="24" t="n"/>
+      <c r="O93" s="27" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="24" t="n"/>
@@ -7419,6 +7609,8 @@
       <c r="K94" s="25" t="n"/>
       <c r="L94" s="24" t="n"/>
       <c r="M94" s="24" t="n"/>
+      <c r="N94" s="24" t="n"/>
+      <c r="O94" s="27" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="24" t="n"/>
@@ -7434,6 +7626,8 @@
       <c r="K95" s="25" t="n"/>
       <c r="L95" s="24" t="n"/>
       <c r="M95" s="24" t="n"/>
+      <c r="N95" s="24" t="n"/>
+      <c r="O95" s="27" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="24" t="n"/>
@@ -7449,6 +7643,8 @@
       <c r="K96" s="25" t="n"/>
       <c r="L96" s="24" t="n"/>
       <c r="M96" s="24" t="n"/>
+      <c r="N96" s="24" t="n"/>
+      <c r="O96" s="27" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="24" t="n"/>
@@ -7464,6 +7660,8 @@
       <c r="K97" s="25" t="n"/>
       <c r="L97" s="24" t="n"/>
       <c r="M97" s="24" t="n"/>
+      <c r="N97" s="24" t="n"/>
+      <c r="O97" s="27" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="24" t="n"/>
@@ -7479,6 +7677,8 @@
       <c r="K98" s="25" t="n"/>
       <c r="L98" s="24" t="n"/>
       <c r="M98" s="24" t="n"/>
+      <c r="N98" s="24" t="n"/>
+      <c r="O98" s="27" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="24" t="n"/>
@@ -7494,6 +7694,8 @@
       <c r="K99" s="25" t="n"/>
       <c r="L99" s="24" t="n"/>
       <c r="M99" s="24" t="n"/>
+      <c r="N99" s="24" t="n"/>
+      <c r="O99" s="27" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="24" t="n"/>
@@ -7509,6 +7711,8 @@
       <c r="K100" s="25" t="n"/>
       <c r="L100" s="24" t="n"/>
       <c r="M100" s="24" t="n"/>
+      <c r="N100" s="24" t="n"/>
+      <c r="O100" s="27" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="24" t="n"/>
@@ -7524,6 +7728,8 @@
       <c r="K101" s="25" t="n"/>
       <c r="L101" s="24" t="n"/>
       <c r="M101" s="24" t="n"/>
+      <c r="N101" s="24" t="n"/>
+      <c r="O101" s="27" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="24" t="n"/>
@@ -7539,6 +7745,8 @@
       <c r="K102" s="25" t="n"/>
       <c r="L102" s="24" t="n"/>
       <c r="M102" s="24" t="n"/>
+      <c r="N102" s="24" t="n"/>
+      <c r="O102" s="27" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="24" t="n"/>
@@ -7554,6 +7762,8 @@
       <c r="K103" s="25" t="n"/>
       <c r="L103" s="24" t="n"/>
       <c r="M103" s="24" t="n"/>
+      <c r="N103" s="24" t="n"/>
+      <c r="O103" s="27" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="24" t="n"/>
@@ -7569,6 +7779,8 @@
       <c r="K104" s="25" t="n"/>
       <c r="L104" s="24" t="n"/>
       <c r="M104" s="24" t="n"/>
+      <c r="N104" s="24" t="n"/>
+      <c r="O104" s="27" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="24" t="n"/>
@@ -7584,6 +7796,8 @@
       <c r="K105" s="25" t="n"/>
       <c r="L105" s="24" t="n"/>
       <c r="M105" s="24" t="n"/>
+      <c r="N105" s="24" t="n"/>
+      <c r="O105" s="27" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="24" t="n"/>
@@ -7599,6 +7813,8 @@
       <c r="K106" s="25" t="n"/>
       <c r="L106" s="24" t="n"/>
       <c r="M106" s="24" t="n"/>
+      <c r="N106" s="24" t="n"/>
+      <c r="O106" s="27" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="24" t="n"/>
@@ -7614,6 +7830,8 @@
       <c r="K107" s="25" t="n"/>
       <c r="L107" s="24" t="n"/>
       <c r="M107" s="24" t="n"/>
+      <c r="N107" s="24" t="n"/>
+      <c r="O107" s="27" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="24" t="n"/>
@@ -7629,6 +7847,8 @@
       <c r="K108" s="25" t="n"/>
       <c r="L108" s="24" t="n"/>
       <c r="M108" s="24" t="n"/>
+      <c r="N108" s="24" t="n"/>
+      <c r="O108" s="27" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="24" t="n"/>
@@ -7644,6 +7864,8 @@
       <c r="K109" s="25" t="n"/>
       <c r="L109" s="24" t="n"/>
       <c r="M109" s="24" t="n"/>
+      <c r="N109" s="24" t="n"/>
+      <c r="O109" s="27" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="24" t="n"/>
@@ -7659,6 +7881,8 @@
       <c r="K110" s="25" t="n"/>
       <c r="L110" s="24" t="n"/>
       <c r="M110" s="24" t="n"/>
+      <c r="N110" s="24" t="n"/>
+      <c r="O110" s="27" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="24" t="n"/>
@@ -7674,6 +7898,8 @@
       <c r="K111" s="25" t="n"/>
       <c r="L111" s="24" t="n"/>
       <c r="M111" s="24" t="n"/>
+      <c r="N111" s="24" t="n"/>
+      <c r="O111" s="27" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="24" t="n"/>
@@ -7689,6 +7915,8 @@
       <c r="K112" s="25" t="n"/>
       <c r="L112" s="24" t="n"/>
       <c r="M112" s="24" t="n"/>
+      <c r="N112" s="24" t="n"/>
+      <c r="O112" s="27" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="24" t="n"/>
@@ -7704,6 +7932,8 @@
       <c r="K113" s="25" t="n"/>
       <c r="L113" s="24" t="n"/>
       <c r="M113" s="24" t="n"/>
+      <c r="N113" s="24" t="n"/>
+      <c r="O113" s="27" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="24" t="n"/>
@@ -7719,6 +7949,8 @@
       <c r="K114" s="25" t="n"/>
       <c r="L114" s="24" t="n"/>
       <c r="M114" s="24" t="n"/>
+      <c r="N114" s="24" t="n"/>
+      <c r="O114" s="27" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="24" t="n"/>
@@ -7734,6 +7966,8 @@
       <c r="K115" s="25" t="n"/>
       <c r="L115" s="24" t="n"/>
       <c r="M115" s="24" t="n"/>
+      <c r="N115" s="24" t="n"/>
+      <c r="O115" s="27" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="24" t="n"/>
@@ -7749,6 +7983,8 @@
       <c r="K116" s="25" t="n"/>
       <c r="L116" s="24" t="n"/>
       <c r="M116" s="24" t="n"/>
+      <c r="N116" s="24" t="n"/>
+      <c r="O116" s="27" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="24" t="n"/>
@@ -7764,6 +8000,8 @@
       <c r="K117" s="25" t="n"/>
       <c r="L117" s="24" t="n"/>
       <c r="M117" s="24" t="n"/>
+      <c r="N117" s="24" t="n"/>
+      <c r="O117" s="27" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="24" t="n"/>
@@ -7779,6 +8017,8 @@
       <c r="K118" s="25" t="n"/>
       <c r="L118" s="24" t="n"/>
       <c r="M118" s="24" t="n"/>
+      <c r="N118" s="24" t="n"/>
+      <c r="O118" s="27" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="24" t="n"/>
@@ -7794,6 +8034,8 @@
       <c r="K119" s="25" t="n"/>
       <c r="L119" s="24" t="n"/>
       <c r="M119" s="24" t="n"/>
+      <c r="N119" s="24" t="n"/>
+      <c r="O119" s="27" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="24" t="n"/>
@@ -7809,6 +8051,8 @@
       <c r="K120" s="25" t="n"/>
       <c r="L120" s="24" t="n"/>
       <c r="M120" s="24" t="n"/>
+      <c r="N120" s="24" t="n"/>
+      <c r="O120" s="27" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="24" t="n"/>
@@ -7824,6 +8068,8 @@
       <c r="K121" s="25" t="n"/>
       <c r="L121" s="24" t="n"/>
       <c r="M121" s="24" t="n"/>
+      <c r="N121" s="24" t="n"/>
+      <c r="O121" s="27" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="24" t="n"/>
@@ -7839,6 +8085,8 @@
       <c r="K122" s="25" t="n"/>
       <c r="L122" s="24" t="n"/>
       <c r="M122" s="24" t="n"/>
+      <c r="N122" s="24" t="n"/>
+      <c r="O122" s="27" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="24" t="n"/>
@@ -7854,6 +8102,8 @@
       <c r="K123" s="25" t="n"/>
       <c r="L123" s="24" t="n"/>
       <c r="M123" s="24" t="n"/>
+      <c r="N123" s="24" t="n"/>
+      <c r="O123" s="27" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="24" t="n"/>
@@ -7869,6 +8119,8 @@
       <c r="K124" s="25" t="n"/>
       <c r="L124" s="24" t="n"/>
       <c r="M124" s="24" t="n"/>
+      <c r="N124" s="24" t="n"/>
+      <c r="O124" s="27" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="24" t="n"/>
@@ -7884,6 +8136,8 @@
       <c r="K125" s="25" t="n"/>
       <c r="L125" s="24" t="n"/>
       <c r="M125" s="24" t="n"/>
+      <c r="N125" s="24" t="n"/>
+      <c r="O125" s="27" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="24" t="n"/>
@@ -7899,6 +8153,8 @@
       <c r="K126" s="25" t="n"/>
       <c r="L126" s="24" t="n"/>
       <c r="M126" s="24" t="n"/>
+      <c r="N126" s="24" t="n"/>
+      <c r="O126" s="27" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="24" t="n"/>
@@ -7914,6 +8170,8 @@
       <c r="K127" s="25" t="n"/>
       <c r="L127" s="24" t="n"/>
       <c r="M127" s="24" t="n"/>
+      <c r="N127" s="24" t="n"/>
+      <c r="O127" s="27" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="24" t="n"/>
@@ -7929,6 +8187,8 @@
       <c r="K128" s="25" t="n"/>
       <c r="L128" s="24" t="n"/>
       <c r="M128" s="24" t="n"/>
+      <c r="N128" s="24" t="n"/>
+      <c r="O128" s="27" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="24" t="n"/>
@@ -7944,6 +8204,8 @@
       <c r="K129" s="25" t="n"/>
       <c r="L129" s="24" t="n"/>
       <c r="M129" s="24" t="n"/>
+      <c r="N129" s="24" t="n"/>
+      <c r="O129" s="27" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="24" t="n"/>
@@ -7959,6 +8221,8 @@
       <c r="K130" s="25" t="n"/>
       <c r="L130" s="24" t="n"/>
       <c r="M130" s="24" t="n"/>
+      <c r="N130" s="24" t="n"/>
+      <c r="O130" s="27" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="24" t="n"/>
@@ -7974,6 +8238,8 @@
       <c r="K131" s="25" t="n"/>
       <c r="L131" s="24" t="n"/>
       <c r="M131" s="24" t="n"/>
+      <c r="N131" s="24" t="n"/>
+      <c r="O131" s="27" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="24" t="n"/>
@@ -7989,6 +8255,8 @@
       <c r="K132" s="25" t="n"/>
       <c r="L132" s="24" t="n"/>
       <c r="M132" s="24" t="n"/>
+      <c r="N132" s="24" t="n"/>
+      <c r="O132" s="27" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="24" t="n"/>
@@ -8004,6 +8272,8 @@
       <c r="K133" s="25" t="n"/>
       <c r="L133" s="24" t="n"/>
       <c r="M133" s="24" t="n"/>
+      <c r="N133" s="24" t="n"/>
+      <c r="O133" s="27" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="24" t="n"/>
@@ -8019,6 +8289,8 @@
       <c r="K134" s="25" t="n"/>
       <c r="L134" s="24" t="n"/>
       <c r="M134" s="24" t="n"/>
+      <c r="N134" s="24" t="n"/>
+      <c r="O134" s="27" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="24" t="n"/>
@@ -8034,6 +8306,8 @@
       <c r="K135" s="25" t="n"/>
       <c r="L135" s="24" t="n"/>
       <c r="M135" s="24" t="n"/>
+      <c r="N135" s="24" t="n"/>
+      <c r="O135" s="27" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="24" t="n"/>
@@ -8049,6 +8323,8 @@
       <c r="K136" s="25" t="n"/>
       <c r="L136" s="24" t="n"/>
       <c r="M136" s="24" t="n"/>
+      <c r="N136" s="24" t="n"/>
+      <c r="O136" s="27" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="24" t="n"/>
@@ -8064,6 +8340,8 @@
       <c r="K137" s="25" t="n"/>
       <c r="L137" s="24" t="n"/>
       <c r="M137" s="24" t="n"/>
+      <c r="N137" s="24" t="n"/>
+      <c r="O137" s="27" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="24" t="n"/>
@@ -8079,6 +8357,8 @@
       <c r="K138" s="25" t="n"/>
       <c r="L138" s="24" t="n"/>
       <c r="M138" s="24" t="n"/>
+      <c r="N138" s="24" t="n"/>
+      <c r="O138" s="27" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="24" t="n"/>
@@ -8094,6 +8374,8 @@
       <c r="K139" s="25" t="n"/>
       <c r="L139" s="24" t="n"/>
       <c r="M139" s="24" t="n"/>
+      <c r="N139" s="24" t="n"/>
+      <c r="O139" s="27" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="24" t="n"/>
@@ -8109,6 +8391,8 @@
       <c r="K140" s="25" t="n"/>
       <c r="L140" s="24" t="n"/>
       <c r="M140" s="24" t="n"/>
+      <c r="N140" s="24" t="n"/>
+      <c r="O140" s="27" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="24" t="n"/>
@@ -8124,6 +8408,8 @@
       <c r="K141" s="25" t="n"/>
       <c r="L141" s="24" t="n"/>
       <c r="M141" s="24" t="n"/>
+      <c r="N141" s="24" t="n"/>
+      <c r="O141" s="27" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="24" t="n"/>
@@ -8139,6 +8425,8 @@
       <c r="K142" s="25" t="n"/>
       <c r="L142" s="24" t="n"/>
       <c r="M142" s="24" t="n"/>
+      <c r="N142" s="24" t="n"/>
+      <c r="O142" s="27" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="24" t="n"/>
@@ -8154,6 +8442,8 @@
       <c r="K143" s="25" t="n"/>
       <c r="L143" s="24" t="n"/>
       <c r="M143" s="24" t="n"/>
+      <c r="N143" s="24" t="n"/>
+      <c r="O143" s="27" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="24" t="n"/>
@@ -8169,6 +8459,8 @@
       <c r="K144" s="25" t="n"/>
       <c r="L144" s="24" t="n"/>
       <c r="M144" s="24" t="n"/>
+      <c r="N144" s="24" t="n"/>
+      <c r="O144" s="27" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="24" t="n"/>
@@ -8184,6 +8476,8 @@
       <c r="K145" s="25" t="n"/>
       <c r="L145" s="24" t="n"/>
       <c r="M145" s="24" t="n"/>
+      <c r="N145" s="24" t="n"/>
+      <c r="O145" s="27" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="24" t="n"/>
@@ -8199,6 +8493,8 @@
       <c r="K146" s="25" t="n"/>
       <c r="L146" s="24" t="n"/>
       <c r="M146" s="24" t="n"/>
+      <c r="N146" s="24" t="n"/>
+      <c r="O146" s="27" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="24" t="n"/>
@@ -8214,6 +8510,8 @@
       <c r="K147" s="25" t="n"/>
       <c r="L147" s="24" t="n"/>
       <c r="M147" s="24" t="n"/>
+      <c r="N147" s="24" t="n"/>
+      <c r="O147" s="27" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="24" t="n"/>
@@ -8229,6 +8527,8 @@
       <c r="K148" s="25" t="n"/>
       <c r="L148" s="24" t="n"/>
       <c r="M148" s="24" t="n"/>
+      <c r="N148" s="24" t="n"/>
+      <c r="O148" s="27" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="24" t="n"/>
@@ -8244,6 +8544,8 @@
       <c r="K149" s="25" t="n"/>
       <c r="L149" s="24" t="n"/>
       <c r="M149" s="24" t="n"/>
+      <c r="N149" s="24" t="n"/>
+      <c r="O149" s="27" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="24" t="n"/>
@@ -8259,6 +8561,8 @@
       <c r="K150" s="25" t="n"/>
       <c r="L150" s="24" t="n"/>
       <c r="M150" s="24" t="n"/>
+      <c r="N150" s="24" t="n"/>
+      <c r="O150" s="27" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="24" t="n"/>
@@ -8274,6 +8578,8 @@
       <c r="K151" s="25" t="n"/>
       <c r="L151" s="24" t="n"/>
       <c r="M151" s="24" t="n"/>
+      <c r="N151" s="24" t="n"/>
+      <c r="O151" s="27" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="24" t="n"/>
@@ -8289,6 +8595,8 @@
       <c r="K152" s="25" t="n"/>
       <c r="L152" s="24" t="n"/>
       <c r="M152" s="24" t="n"/>
+      <c r="N152" s="24" t="n"/>
+      <c r="O152" s="27" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="24" t="n"/>
@@ -8304,6 +8612,8 @@
       <c r="K153" s="25" t="n"/>
       <c r="L153" s="24" t="n"/>
       <c r="M153" s="24" t="n"/>
+      <c r="N153" s="24" t="n"/>
+      <c r="O153" s="27" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="24" t="n"/>
@@ -8319,6 +8629,8 @@
       <c r="K154" s="25" t="n"/>
       <c r="L154" s="24" t="n"/>
       <c r="M154" s="24" t="n"/>
+      <c r="N154" s="24" t="n"/>
+      <c r="O154" s="27" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="24" t="n"/>
@@ -8334,6 +8646,8 @@
       <c r="K155" s="25" t="n"/>
       <c r="L155" s="24" t="n"/>
       <c r="M155" s="24" t="n"/>
+      <c r="N155" s="24" t="n"/>
+      <c r="O155" s="27" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="24" t="n"/>
@@ -8349,6 +8663,8 @@
       <c r="K156" s="25" t="n"/>
       <c r="L156" s="24" t="n"/>
       <c r="M156" s="24" t="n"/>
+      <c r="N156" s="24" t="n"/>
+      <c r="O156" s="27" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="24" t="n"/>
@@ -8364,6 +8680,8 @@
       <c r="K157" s="25" t="n"/>
       <c r="L157" s="24" t="n"/>
       <c r="M157" s="24" t="n"/>
+      <c r="N157" s="24" t="n"/>
+      <c r="O157" s="27" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="24" t="n"/>
@@ -8379,6 +8697,8 @@
       <c r="K158" s="25" t="n"/>
       <c r="L158" s="24" t="n"/>
       <c r="M158" s="24" t="n"/>
+      <c r="N158" s="24" t="n"/>
+      <c r="O158" s="27" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="24" t="n"/>
@@ -8394,6 +8714,8 @@
       <c r="K159" s="25" t="n"/>
       <c r="L159" s="24" t="n"/>
       <c r="M159" s="24" t="n"/>
+      <c r="N159" s="24" t="n"/>
+      <c r="O159" s="27" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="24" t="n"/>
@@ -8409,6 +8731,8 @@
       <c r="K160" s="25" t="n"/>
       <c r="L160" s="24" t="n"/>
       <c r="M160" s="24" t="n"/>
+      <c r="N160" s="24" t="n"/>
+      <c r="O160" s="27" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="24" t="n"/>
@@ -8424,6 +8748,8 @@
       <c r="K161" s="25" t="n"/>
       <c r="L161" s="24" t="n"/>
       <c r="M161" s="24" t="n"/>
+      <c r="N161" s="24" t="n"/>
+      <c r="O161" s="27" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="24" t="n"/>
@@ -8439,6 +8765,8 @@
       <c r="K162" s="25" t="n"/>
       <c r="L162" s="24" t="n"/>
       <c r="M162" s="24" t="n"/>
+      <c r="N162" s="24" t="n"/>
+      <c r="O162" s="27" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="24" t="n"/>
@@ -8454,6 +8782,8 @@
       <c r="K163" s="25" t="n"/>
       <c r="L163" s="24" t="n"/>
       <c r="M163" s="24" t="n"/>
+      <c r="N163" s="24" t="n"/>
+      <c r="O163" s="27" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="24" t="n"/>
@@ -8469,6 +8799,8 @@
       <c r="K164" s="25" t="n"/>
       <c r="L164" s="24" t="n"/>
       <c r="M164" s="24" t="n"/>
+      <c r="N164" s="24" t="n"/>
+      <c r="O164" s="27" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="24" t="n"/>
@@ -8484,6 +8816,8 @@
       <c r="K165" s="25" t="n"/>
       <c r="L165" s="24" t="n"/>
       <c r="M165" s="24" t="n"/>
+      <c r="N165" s="24" t="n"/>
+      <c r="O165" s="27" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="24" t="n"/>
@@ -8499,6 +8833,8 @@
       <c r="K166" s="25" t="n"/>
       <c r="L166" s="24" t="n"/>
       <c r="M166" s="24" t="n"/>
+      <c r="N166" s="24" t="n"/>
+      <c r="O166" s="27" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="24" t="n"/>
@@ -8514,6 +8850,8 @@
       <c r="K167" s="25" t="n"/>
       <c r="L167" s="24" t="n"/>
       <c r="M167" s="24" t="n"/>
+      <c r="N167" s="24" t="n"/>
+      <c r="O167" s="27" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="24" t="n"/>
@@ -8529,6 +8867,8 @@
       <c r="K168" s="25" t="n"/>
       <c r="L168" s="24" t="n"/>
       <c r="M168" s="24" t="n"/>
+      <c r="N168" s="24" t="n"/>
+      <c r="O168" s="27" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="24" t="n"/>
@@ -8544,6 +8884,8 @@
       <c r="K169" s="25" t="n"/>
       <c r="L169" s="24" t="n"/>
       <c r="M169" s="24" t="n"/>
+      <c r="N169" s="24" t="n"/>
+      <c r="O169" s="27" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="24" t="n"/>
@@ -8559,6 +8901,8 @@
       <c r="K170" s="25" t="n"/>
       <c r="L170" s="24" t="n"/>
       <c r="M170" s="24" t="n"/>
+      <c r="N170" s="24" t="n"/>
+      <c r="O170" s="27" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="24" t="n"/>
@@ -8574,6 +8918,8 @@
       <c r="K171" s="25" t="n"/>
       <c r="L171" s="24" t="n"/>
       <c r="M171" s="24" t="n"/>
+      <c r="N171" s="24" t="n"/>
+      <c r="O171" s="27" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="24" t="n"/>
@@ -8589,6 +8935,8 @@
       <c r="K172" s="25" t="n"/>
       <c r="L172" s="24" t="n"/>
       <c r="M172" s="24" t="n"/>
+      <c r="N172" s="24" t="n"/>
+      <c r="O172" s="27" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="24" t="n"/>
@@ -8604,6 +8952,8 @@
       <c r="K173" s="25" t="n"/>
       <c r="L173" s="24" t="n"/>
       <c r="M173" s="24" t="n"/>
+      <c r="N173" s="24" t="n"/>
+      <c r="O173" s="27" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="24" t="n"/>
@@ -8619,6 +8969,8 @@
       <c r="K174" s="25" t="n"/>
       <c r="L174" s="24" t="n"/>
       <c r="M174" s="24" t="n"/>
+      <c r="N174" s="24" t="n"/>
+      <c r="O174" s="27" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="24" t="n"/>
@@ -8634,6 +8986,8 @@
       <c r="K175" s="25" t="n"/>
       <c r="L175" s="24" t="n"/>
       <c r="M175" s="24" t="n"/>
+      <c r="N175" s="24" t="n"/>
+      <c r="O175" s="27" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="24" t="n"/>
@@ -8649,6 +9003,8 @@
       <c r="K176" s="25" t="n"/>
       <c r="L176" s="24" t="n"/>
       <c r="M176" s="24" t="n"/>
+      <c r="N176" s="24" t="n"/>
+      <c r="O176" s="27" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="24" t="n"/>
@@ -8664,6 +9020,8 @@
       <c r="K177" s="25" t="n"/>
       <c r="L177" s="24" t="n"/>
       <c r="M177" s="24" t="n"/>
+      <c r="N177" s="24" t="n"/>
+      <c r="O177" s="27" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="24" t="n"/>
@@ -8679,6 +9037,8 @@
       <c r="K178" s="25" t="n"/>
       <c r="L178" s="24" t="n"/>
       <c r="M178" s="24" t="n"/>
+      <c r="N178" s="24" t="n"/>
+      <c r="O178" s="27" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="24" t="n"/>
@@ -8694,6 +9054,8 @@
       <c r="K179" s="25" t="n"/>
       <c r="L179" s="24" t="n"/>
       <c r="M179" s="24" t="n"/>
+      <c r="N179" s="24" t="n"/>
+      <c r="O179" s="27" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="24" t="n"/>
@@ -8709,6 +9071,8 @@
       <c r="K180" s="25" t="n"/>
       <c r="L180" s="24" t="n"/>
       <c r="M180" s="24" t="n"/>
+      <c r="N180" s="24" t="n"/>
+      <c r="O180" s="27" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="24" t="n"/>
@@ -8724,6 +9088,8 @@
       <c r="K181" s="25" t="n"/>
       <c r="L181" s="24" t="n"/>
       <c r="M181" s="24" t="n"/>
+      <c r="N181" s="24" t="n"/>
+      <c r="O181" s="27" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="24" t="n"/>
@@ -8739,6 +9105,8 @@
       <c r="K182" s="25" t="n"/>
       <c r="L182" s="24" t="n"/>
       <c r="M182" s="24" t="n"/>
+      <c r="N182" s="24" t="n"/>
+      <c r="O182" s="27" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="24" t="n"/>
@@ -8754,6 +9122,8 @@
       <c r="K183" s="25" t="n"/>
       <c r="L183" s="24" t="n"/>
       <c r="M183" s="24" t="n"/>
+      <c r="N183" s="24" t="n"/>
+      <c r="O183" s="27" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="24" t="n"/>
@@ -8769,6 +9139,8 @@
       <c r="K184" s="25" t="n"/>
       <c r="L184" s="24" t="n"/>
       <c r="M184" s="24" t="n"/>
+      <c r="N184" s="24" t="n"/>
+      <c r="O184" s="27" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="24" t="n"/>
@@ -8784,6 +9156,8 @@
       <c r="K185" s="25" t="n"/>
       <c r="L185" s="24" t="n"/>
       <c r="M185" s="24" t="n"/>
+      <c r="N185" s="24" t="n"/>
+      <c r="O185" s="27" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="24" t="n"/>
@@ -8799,6 +9173,8 @@
       <c r="K186" s="25" t="n"/>
       <c r="L186" s="24" t="n"/>
       <c r="M186" s="24" t="n"/>
+      <c r="N186" s="24" t="n"/>
+      <c r="O186" s="27" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="24" t="n"/>
@@ -8814,6 +9190,8 @@
       <c r="K187" s="25" t="n"/>
       <c r="L187" s="24" t="n"/>
       <c r="M187" s="24" t="n"/>
+      <c r="N187" s="24" t="n"/>
+      <c r="O187" s="27" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="24" t="n"/>
@@ -8829,6 +9207,8 @@
       <c r="K188" s="25" t="n"/>
       <c r="L188" s="24" t="n"/>
       <c r="M188" s="24" t="n"/>
+      <c r="N188" s="24" t="n"/>
+      <c r="O188" s="27" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="24" t="n"/>
@@ -8844,6 +9224,8 @@
       <c r="K189" s="25" t="n"/>
       <c r="L189" s="24" t="n"/>
       <c r="M189" s="24" t="n"/>
+      <c r="N189" s="24" t="n"/>
+      <c r="O189" s="27" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="24" t="n"/>
@@ -8859,6 +9241,8 @@
       <c r="K190" s="25" t="n"/>
       <c r="L190" s="24" t="n"/>
       <c r="M190" s="24" t="n"/>
+      <c r="N190" s="24" t="n"/>
+      <c r="O190" s="27" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="24" t="n"/>
@@ -8874,6 +9258,8 @@
       <c r="K191" s="25" t="n"/>
       <c r="L191" s="24" t="n"/>
       <c r="M191" s="24" t="n"/>
+      <c r="N191" s="24" t="n"/>
+      <c r="O191" s="27" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="24" t="n"/>
@@ -8889,6 +9275,8 @@
       <c r="K192" s="25" t="n"/>
       <c r="L192" s="24" t="n"/>
       <c r="M192" s="24" t="n"/>
+      <c r="N192" s="24" t="n"/>
+      <c r="O192" s="27" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="24" t="n"/>
@@ -8904,6 +9292,8 @@
       <c r="K193" s="25" t="n"/>
       <c r="L193" s="24" t="n"/>
       <c r="M193" s="24" t="n"/>
+      <c r="N193" s="24" t="n"/>
+      <c r="O193" s="27" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="24" t="n"/>
@@ -8919,6 +9309,8 @@
       <c r="K194" s="25" t="n"/>
       <c r="L194" s="24" t="n"/>
       <c r="M194" s="24" t="n"/>
+      <c r="N194" s="24" t="n"/>
+      <c r="O194" s="27" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="24" t="n"/>
@@ -8934,6 +9326,8 @@
       <c r="K195" s="25" t="n"/>
       <c r="L195" s="24" t="n"/>
       <c r="M195" s="24" t="n"/>
+      <c r="N195" s="24" t="n"/>
+      <c r="O195" s="27" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="24" t="n"/>
@@ -8949,6 +9343,8 @@
       <c r="K196" s="25" t="n"/>
       <c r="L196" s="24" t="n"/>
       <c r="M196" s="24" t="n"/>
+      <c r="N196" s="24" t="n"/>
+      <c r="O196" s="27" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="24" t="n"/>
@@ -8964,6 +9360,8 @@
       <c r="K197" s="25" t="n"/>
       <c r="L197" s="24" t="n"/>
       <c r="M197" s="24" t="n"/>
+      <c r="N197" s="24" t="n"/>
+      <c r="O197" s="27" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="24" t="n"/>
@@ -8979,6 +9377,8 @@
       <c r="K198" s="25" t="n"/>
       <c r="L198" s="24" t="n"/>
       <c r="M198" s="24" t="n"/>
+      <c r="N198" s="24" t="n"/>
+      <c r="O198" s="27" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="24" t="n"/>
@@ -8994,6 +9394,8 @@
       <c r="K199" s="25" t="n"/>
       <c r="L199" s="24" t="n"/>
       <c r="M199" s="24" t="n"/>
+      <c r="N199" s="24" t="n"/>
+      <c r="O199" s="27" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="24" t="n"/>
@@ -9009,6 +9411,8 @@
       <c r="K200" s="25" t="n"/>
       <c r="L200" s="24" t="n"/>
       <c r="M200" s="24" t="n"/>
+      <c r="N200" s="24" t="n"/>
+      <c r="O200" s="27" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="24" t="n"/>
@@ -9024,6 +9428,8 @@
       <c r="K201" s="25" t="n"/>
       <c r="L201" s="24" t="n"/>
       <c r="M201" s="24" t="n"/>
+      <c r="N201" s="24" t="n"/>
+      <c r="O201" s="27" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="24" t="n"/>
@@ -9039,6 +9445,8 @@
       <c r="K202" s="25" t="n"/>
       <c r="L202" s="24" t="n"/>
       <c r="M202" s="24" t="n"/>
+      <c r="N202" s="24" t="n"/>
+      <c r="O202" s="27" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="24" t="n"/>
@@ -9054,6 +9462,8 @@
       <c r="K203" s="25" t="n"/>
       <c r="L203" s="24" t="n"/>
       <c r="M203" s="24" t="n"/>
+      <c r="N203" s="24" t="n"/>
+      <c r="O203" s="27" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="24" t="n"/>
@@ -9069,6 +9479,8 @@
       <c r="K204" s="25" t="n"/>
       <c r="L204" s="24" t="n"/>
       <c r="M204" s="24" t="n"/>
+      <c r="N204" s="24" t="n"/>
+      <c r="O204" s="27" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="24" t="n"/>
@@ -9084,6 +9496,8 @@
       <c r="K205" s="25" t="n"/>
       <c r="L205" s="24" t="n"/>
       <c r="M205" s="24" t="n"/>
+      <c r="N205" s="24" t="n"/>
+      <c r="O205" s="27" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="24" t="n"/>
@@ -9099,6 +9513,8 @@
       <c r="K206" s="25" t="n"/>
       <c r="L206" s="24" t="n"/>
       <c r="M206" s="24" t="n"/>
+      <c r="N206" s="24" t="n"/>
+      <c r="O206" s="27" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="24" t="n"/>
@@ -9114,6 +9530,8 @@
       <c r="K207" s="25" t="n"/>
       <c r="L207" s="24" t="n"/>
       <c r="M207" s="24" t="n"/>
+      <c r="N207" s="24" t="n"/>
+      <c r="O207" s="27" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="24" t="n"/>
@@ -9129,6 +9547,8 @@
       <c r="K208" s="25" t="n"/>
       <c r="L208" s="24" t="n"/>
       <c r="M208" s="24" t="n"/>
+      <c r="N208" s="24" t="n"/>
+      <c r="O208" s="27" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="24" t="n"/>
@@ -9144,6 +9564,8 @@
       <c r="K209" s="25" t="n"/>
       <c r="L209" s="24" t="n"/>
       <c r="M209" s="24" t="n"/>
+      <c r="N209" s="24" t="n"/>
+      <c r="O209" s="27" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="24" t="n"/>
@@ -9159,6 +9581,8 @@
       <c r="K210" s="25" t="n"/>
       <c r="L210" s="24" t="n"/>
       <c r="M210" s="24" t="n"/>
+      <c r="N210" s="24" t="n"/>
+      <c r="O210" s="27" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="24" t="n"/>
@@ -9174,6 +9598,8 @@
       <c r="K211" s="25" t="n"/>
       <c r="L211" s="24" t="n"/>
       <c r="M211" s="24" t="n"/>
+      <c r="N211" s="24" t="n"/>
+      <c r="O211" s="27" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="24" t="n"/>
@@ -9189,6 +9615,8 @@
       <c r="K212" s="25" t="n"/>
       <c r="L212" s="24" t="n"/>
       <c r="M212" s="24" t="n"/>
+      <c r="N212" s="24" t="n"/>
+      <c r="O212" s="27" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="24" t="n"/>
@@ -9204,6 +9632,8 @@
       <c r="K213" s="25" t="n"/>
       <c r="L213" s="24" t="n"/>
       <c r="M213" s="24" t="n"/>
+      <c r="N213" s="24" t="n"/>
+      <c r="O213" s="27" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="24" t="n"/>
@@ -9219,6 +9649,8 @@
       <c r="K214" s="25" t="n"/>
       <c r="L214" s="24" t="n"/>
       <c r="M214" s="24" t="n"/>
+      <c r="N214" s="24" t="n"/>
+      <c r="O214" s="27" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="24" t="n"/>
@@ -9234,6 +9666,8 @@
       <c r="K215" s="25" t="n"/>
       <c r="L215" s="24" t="n"/>
       <c r="M215" s="24" t="n"/>
+      <c r="N215" s="24" t="n"/>
+      <c r="O215" s="27" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="24" t="n"/>
@@ -9249,6 +9683,8 @@
       <c r="K216" s="25" t="n"/>
       <c r="L216" s="24" t="n"/>
       <c r="M216" s="24" t="n"/>
+      <c r="N216" s="24" t="n"/>
+      <c r="O216" s="27" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="24" t="n"/>
@@ -9264,6 +9700,8 @@
       <c r="K217" s="25" t="n"/>
       <c r="L217" s="24" t="n"/>
       <c r="M217" s="24" t="n"/>
+      <c r="N217" s="24" t="n"/>
+      <c r="O217" s="27" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="24" t="n"/>
@@ -9279,6 +9717,8 @@
       <c r="K218" s="25" t="n"/>
       <c r="L218" s="24" t="n"/>
       <c r="M218" s="24" t="n"/>
+      <c r="N218" s="24" t="n"/>
+      <c r="O218" s="27" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="24" t="n"/>
@@ -9294,6 +9734,8 @@
       <c r="K219" s="25" t="n"/>
       <c r="L219" s="24" t="n"/>
       <c r="M219" s="24" t="n"/>
+      <c r="N219" s="24" t="n"/>
+      <c r="O219" s="27" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="24" t="n"/>
@@ -9309,6 +9751,8 @@
       <c r="K220" s="25" t="n"/>
       <c r="L220" s="24" t="n"/>
       <c r="M220" s="24" t="n"/>
+      <c r="N220" s="24" t="n"/>
+      <c r="O220" s="27" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="24" t="n"/>
@@ -9324,6 +9768,8 @@
       <c r="K221" s="25" t="n"/>
       <c r="L221" s="24" t="n"/>
       <c r="M221" s="24" t="n"/>
+      <c r="N221" s="24" t="n"/>
+      <c r="O221" s="27" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="24" t="n"/>
@@ -9339,6 +9785,8 @@
       <c r="K222" s="25" t="n"/>
       <c r="L222" s="24" t="n"/>
       <c r="M222" s="24" t="n"/>
+      <c r="N222" s="24" t="n"/>
+      <c r="O222" s="27" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="24" t="n"/>
@@ -9354,6 +9802,8 @@
       <c r="K223" s="25" t="n"/>
       <c r="L223" s="24" t="n"/>
       <c r="M223" s="24" t="n"/>
+      <c r="N223" s="24" t="n"/>
+      <c r="O223" s="27" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="24" t="n"/>
@@ -9369,6 +9819,8 @@
       <c r="K224" s="25" t="n"/>
       <c r="L224" s="24" t="n"/>
       <c r="M224" s="24" t="n"/>
+      <c r="N224" s="24" t="n"/>
+      <c r="O224" s="27" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="24" t="n"/>
@@ -9384,6 +9836,8 @@
       <c r="K225" s="25" t="n"/>
       <c r="L225" s="24" t="n"/>
       <c r="M225" s="24" t="n"/>
+      <c r="N225" s="24" t="n"/>
+      <c r="O225" s="27" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="24" t="n"/>
@@ -9399,6 +9853,8 @@
       <c r="K226" s="25" t="n"/>
       <c r="L226" s="24" t="n"/>
       <c r="M226" s="24" t="n"/>
+      <c r="N226" s="24" t="n"/>
+      <c r="O226" s="27" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="24" t="n"/>
@@ -9414,6 +9870,8 @@
       <c r="K227" s="25" t="n"/>
       <c r="L227" s="24" t="n"/>
       <c r="M227" s="24" t="n"/>
+      <c r="N227" s="24" t="n"/>
+      <c r="O227" s="27" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="24" t="n"/>
@@ -9429,6 +9887,8 @@
       <c r="K228" s="25" t="n"/>
       <c r="L228" s="24" t="n"/>
       <c r="M228" s="24" t="n"/>
+      <c r="N228" s="24" t="n"/>
+      <c r="O228" s="27" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="24" t="n"/>
@@ -9444,6 +9904,8 @@
       <c r="K229" s="25" t="n"/>
       <c r="L229" s="24" t="n"/>
       <c r="M229" s="24" t="n"/>
+      <c r="N229" s="24" t="n"/>
+      <c r="O229" s="27" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="24" t="n"/>
@@ -9459,6 +9921,8 @@
       <c r="K230" s="25" t="n"/>
       <c r="L230" s="24" t="n"/>
       <c r="M230" s="24" t="n"/>
+      <c r="N230" s="24" t="n"/>
+      <c r="O230" s="27" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="24" t="n"/>
@@ -9474,6 +9938,8 @@
       <c r="K231" s="25" t="n"/>
       <c r="L231" s="24" t="n"/>
       <c r="M231" s="24" t="n"/>
+      <c r="N231" s="24" t="n"/>
+      <c r="O231" s="27" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="24" t="n"/>
@@ -9489,6 +9955,8 @@
       <c r="K232" s="25" t="n"/>
       <c r="L232" s="24" t="n"/>
       <c r="M232" s="24" t="n"/>
+      <c r="N232" s="24" t="n"/>
+      <c r="O232" s="27" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="24" t="n"/>
@@ -9504,6 +9972,8 @@
       <c r="K233" s="25" t="n"/>
       <c r="L233" s="24" t="n"/>
       <c r="M233" s="24" t="n"/>
+      <c r="N233" s="24" t="n"/>
+      <c r="O233" s="27" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="24" t="n"/>
@@ -9519,6 +9989,8 @@
       <c r="K234" s="25" t="n"/>
       <c r="L234" s="24" t="n"/>
       <c r="M234" s="24" t="n"/>
+      <c r="N234" s="24" t="n"/>
+      <c r="O234" s="27" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="24" t="n"/>
@@ -9534,6 +10006,8 @@
       <c r="K235" s="25" t="n"/>
       <c r="L235" s="24" t="n"/>
       <c r="M235" s="24" t="n"/>
+      <c r="N235" s="24" t="n"/>
+      <c r="O235" s="27" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="24" t="n"/>
@@ -9549,6 +10023,8 @@
       <c r="K236" s="25" t="n"/>
       <c r="L236" s="24" t="n"/>
       <c r="M236" s="24" t="n"/>
+      <c r="N236" s="24" t="n"/>
+      <c r="O236" s="27" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="24" t="n"/>
@@ -9564,6 +10040,8 @@
       <c r="K237" s="25" t="n"/>
       <c r="L237" s="24" t="n"/>
       <c r="M237" s="24" t="n"/>
+      <c r="N237" s="24" t="n"/>
+      <c r="O237" s="27" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="24" t="n"/>
@@ -9579,6 +10057,8 @@
       <c r="K238" s="25" t="n"/>
       <c r="L238" s="24" t="n"/>
       <c r="M238" s="24" t="n"/>
+      <c r="N238" s="24" t="n"/>
+      <c r="O238" s="27" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="24" t="n"/>
@@ -9594,6 +10074,8 @@
       <c r="K239" s="25" t="n"/>
       <c r="L239" s="24" t="n"/>
       <c r="M239" s="24" t="n"/>
+      <c r="N239" s="24" t="n"/>
+      <c r="O239" s="27" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="24" t="n"/>
@@ -9609,6 +10091,8 @@
       <c r="K240" s="25" t="n"/>
       <c r="L240" s="24" t="n"/>
       <c r="M240" s="24" t="n"/>
+      <c r="N240" s="24" t="n"/>
+      <c r="O240" s="27" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="24" t="n"/>
@@ -9624,6 +10108,8 @@
       <c r="K241" s="25" t="n"/>
       <c r="L241" s="24" t="n"/>
       <c r="M241" s="24" t="n"/>
+      <c r="N241" s="24" t="n"/>
+      <c r="O241" s="27" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="24" t="n"/>
@@ -9639,6 +10125,8 @@
       <c r="K242" s="25" t="n"/>
       <c r="L242" s="24" t="n"/>
       <c r="M242" s="24" t="n"/>
+      <c r="N242" s="24" t="n"/>
+      <c r="O242" s="27" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="24" t="n"/>
@@ -9654,6 +10142,8 @@
       <c r="K243" s="25" t="n"/>
       <c r="L243" s="24" t="n"/>
       <c r="M243" s="24" t="n"/>
+      <c r="N243" s="24" t="n"/>
+      <c r="O243" s="27" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="24" t="n"/>
@@ -9669,6 +10159,8 @@
       <c r="K244" s="25" t="n"/>
       <c r="L244" s="24" t="n"/>
       <c r="M244" s="24" t="n"/>
+      <c r="N244" s="24" t="n"/>
+      <c r="O244" s="27" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="24" t="n"/>
@@ -9684,6 +10176,8 @@
       <c r="K245" s="25" t="n"/>
       <c r="L245" s="24" t="n"/>
       <c r="M245" s="24" t="n"/>
+      <c r="N245" s="24" t="n"/>
+      <c r="O245" s="27" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="24" t="n"/>
@@ -9699,6 +10193,8 @@
       <c r="K246" s="25" t="n"/>
       <c r="L246" s="24" t="n"/>
       <c r="M246" s="24" t="n"/>
+      <c r="N246" s="24" t="n"/>
+      <c r="O246" s="27" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="24" t="n"/>
@@ -9714,6 +10210,8 @@
       <c r="K247" s="25" t="n"/>
       <c r="L247" s="24" t="n"/>
       <c r="M247" s="24" t="n"/>
+      <c r="N247" s="24" t="n"/>
+      <c r="O247" s="27" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="24" t="n"/>
@@ -9729,6 +10227,8 @@
       <c r="K248" s="25" t="n"/>
       <c r="L248" s="24" t="n"/>
       <c r="M248" s="24" t="n"/>
+      <c r="N248" s="24" t="n"/>
+      <c r="O248" s="27" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="24" t="n"/>
@@ -9744,6 +10244,8 @@
       <c r="K249" s="25" t="n"/>
       <c r="L249" s="24" t="n"/>
       <c r="M249" s="24" t="n"/>
+      <c r="N249" s="24" t="n"/>
+      <c r="O249" s="27" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="24" t="n"/>
@@ -9759,6 +10261,8 @@
       <c r="K250" s="25" t="n"/>
       <c r="L250" s="24" t="n"/>
       <c r="M250" s="24" t="n"/>
+      <c r="N250" s="24" t="n"/>
+      <c r="O250" s="27" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="24" t="n"/>
@@ -9774,6 +10278,8 @@
       <c r="K251" s="25" t="n"/>
       <c r="L251" s="24" t="n"/>
       <c r="M251" s="24" t="n"/>
+      <c r="N251" s="24" t="n"/>
+      <c r="O251" s="27" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="24" t="n"/>
@@ -9789,6 +10295,8 @@
       <c r="K252" s="25" t="n"/>
       <c r="L252" s="24" t="n"/>
       <c r="M252" s="24" t="n"/>
+      <c r="N252" s="24" t="n"/>
+      <c r="O252" s="27" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="24" t="n"/>
@@ -9804,6 +10312,8 @@
       <c r="K253" s="25" t="n"/>
       <c r="L253" s="24" t="n"/>
       <c r="M253" s="24" t="n"/>
+      <c r="N253" s="24" t="n"/>
+      <c r="O253" s="27" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="24" t="n"/>
@@ -9819,15 +10329,22 @@
       <c r="K254" s="25" t="n"/>
       <c r="L254" s="24" t="n"/>
       <c r="M254" s="24" t="n"/>
+      <c r="N254" s="24" t="n"/>
+      <c r="O254" s="27" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:M254">
+  <conditionalFormatting sqref="A5:O254">
     <cfRule type="expression" priority="1" dxfId="2" stopIfTrue="0">
       <formula>$H5="Odmítnuto"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O254">
+    <cfRule type="expression" priority="2" dxfId="4" stopIfTrue="0">
+      <formula>$O5="Ano"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H5:H254">
-    <cfRule type="expression" priority="2" dxfId="4" stopIfTrue="0">
+    <cfRule type="expression" priority="3" dxfId="4" stopIfTrue="0">
       <formula>$H5="Potvrzeno"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9841,7 +10358,7 @@
     <dataValidation sqref="F5:F254" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Neplatná hodnota" error="Vyberte hodnotu ze seznamu." type="list">
       <formula1>"Obřad a hostina,Jen večer,Jen oznámení"</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G254 J5:J254" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Neplatná hodnota" error="Vyberte hodnotu ze seznamu." type="list">
+    <dataValidation sqref="G5:G254 J5:J254 O5:O254" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Neplatná hodnota" error="Vyberte hodnotu ze seznamu." type="list">
       <formula1>"Ano,Ne"</formula1>
     </dataValidation>
     <dataValidation sqref="H5:H254" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Neplatná hodnota" error="Vyberte hodnotu ze seznamu." type="list">
@@ -11780,7 +12297,7 @@
     <row r="8">
       <c r="B8" s="43" t="inlineStr">
         <is>
-          <t>4. Hosté: jeden řádek = jedna pozvánka. Do sloupce Osob napište, kolik lidí na ni přijde.</t>
+          <t>4. Hosté: jeden řádek = jedna pozvánka. Do sloupce Osob napište, kolik lidí na ni přijde. Po svatbě si tu zapíšete dary a komu už jste poděkovali.</t>
         </is>
       </c>
     </row>
@@ -11876,7 +12393,7 @@
     <row r="24">
       <c r="B24" s="38" t="inlineStr">
         <is>
-          <t>Ano, beru · anoberu.cz · verze 1.0</t>
+          <t>Ano, beru · anoberu.cz · verze 1.1</t>
         </is>
       </c>
     </row>

</xml_diff>